<commit_message>
Simplify portfolio upload template
</commit_message>
<xml_diff>
--- a/docs/portfolio_template.xlsx
+++ b/docs/portfolio_template.xlsx
@@ -2,8 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Raba6bdab62834082"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portefeuille" sheetId="2" r:id="R199f66f7118d4321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portefeuille" sheetId="1" r:id="R6a91ec12cb6749a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -194,123 +193,61 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Modele portefeuille - eaux souterraines</x:v>
+        <x:v>siret</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Mode d'emploi</x:v>
+      </x:c>
+      <x:c r="D1" t="str"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>12345678901234</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Champ cle</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>siret</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Remplis la feuille Portefeuille avec une ligne par site ou etablissement. Seule la colonne siret est indispensable pour la premiere version.</x:v>
+        <x:v>98765432109876</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Obligatoire</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>oui</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>11111111111111</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Format</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>14 chiffres</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>Colonnes attendues</x:v>
+      <x:c r="C5" t="str">
+        <x:v>Le reste</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>deduit automatiquement si le SIRET matche un site ICPE</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>portfolio_name</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>Nom du portefeuille, de la business unit ou du contrat</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>company_name</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>Nom lisible de la societe</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>siret</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>SIRET a 14 chiffres</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>site_label</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>Nom du site ou etiquette interne facultative</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>notes</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>Champ libre facultatif</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" t="str">
-        <x:v>portfolio_name</x:v>
-      </x:c>
-      <x:c r="B1" t="str">
-        <x:v>company_name</x:v>
-      </x:c>
-      <x:c r="C1" t="str">
-        <x:v>siret</x:v>
-      </x:c>
-      <x:c r="D1" t="str">
-        <x:v>site_label</x:v>
-      </x:c>
-      <x:c r="E1" t="str">
-        <x:v>notes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>Portefeuille demo</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>Societe Exemple A</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>12345678901234</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
-        <x:v>Usine Nord</x:v>
-      </x:c>
-      <x:c r="E2" t="str">
-        <x:v>Remplacer cette ligne</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>Portefeuille demo</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>Societe Exemple B</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>98765432109876</x:v>
-      </x:c>
-      <x:c r="D3" t="str">
-        <x:v>Entrepot Ouest</x:v>
-      </x:c>
-      <x:c r="E3" t="str"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str"/>
-      <x:c r="B4" t="str"/>
-      <x:c r="C4" t="str"/>
-      <x:c r="D4" t="str"/>
-      <x:c r="E4" t="str"/>
+      <x:c r="C6" t="str">
+        <x:v>Exemples</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Les lignes 2 a 4 peuvent etre supprimees</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>